<commit_message>
chore: hands-on update - remove Japanese from data, add result_artifacts examples
- Fixture/configs: replace Japanese column names with English
  (LineNo, Item, Qty, Extra1, Extra2, Note, Date)
- Templates: add result_artifacts with labels
  (import_excel_region: read/df 'Detail table', export_excel_region: write/bytes 'Excel file')
- Hands-on: display full result_artifacts list with labels in verify steps

Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/tests/fixtures/excel/test_detect_region_input.xlsx
+++ b/tests/fixtures/excel/test_detect_region_input.xlsx
@@ -467,37 +467,37 @@
     <row r="6">
       <c r="B6" t="inlineStr">
         <is>
-          <t>明細No</t>
+          <t>LineNo</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>品名</t>
+          <t>Item</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>数量</t>
+          <t>Qty</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>余計1</t>
+          <t>Extra1</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>余計2</t>
+          <t>Extra2</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>備考</t>
+          <t>Note</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>日付</t>
+          <t>Date</t>
         </is>
       </c>
     </row>

</xml_diff>